<commit_message>
- Se crea SIGMA_PRUEBAS_S1-md como evidencia de las pruebas realizadas - Informe de pruebas (word) https://claude.ai/code/artifact/768a2676-4131-4d5d-ba7e-fb382fa7c23e?open_in_browser=1
</commit_message>
<xml_diff>
--- a/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S1.xlsx
+++ b/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Capstone\SIGMA\Fase 2\Sprint Backlogs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CAPSTONE\Fase 2\Sprint Backlogs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF33AB52-D91C-44FC-93E6-F68153EF70B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14D6C4A8-3020-4D16-BF71-7189CB90599A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sprint" sheetId="1" r:id="rId1"/>
@@ -2934,18 +2934,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
@@ -3450,7 +3450,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B6:H58"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
     <col min="2" max="2" width="32" customWidth="1"/>
@@ -3458,39 +3458,39 @@
     <col min="7" max="8" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="6" spans="2:8" ht="23.4" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:8" ht="23.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B7" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B10" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="26" t="s">
+    <row r="11" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="C11" s="27"/>
-      <c r="D11" s="27"/>
-      <c r="E11" s="27"/>
-      <c r="F11" s="27"/>
-      <c r="G11" s="27"/>
-      <c r="H11" s="27"/>
-    </row>
-    <row r="12" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="28"/>
+      <c r="C11" s="26"/>
+      <c r="D11" s="26"/>
+      <c r="E11" s="26"/>
+      <c r="F11" s="26"/>
+      <c r="G11" s="26"/>
+      <c r="H11" s="26"/>
+    </row>
+    <row r="12" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="27"/>
       <c r="C12" s="24"/>
       <c r="D12" s="24"/>
       <c r="E12" s="24"/>
@@ -3498,8 +3498,8 @@
       <c r="G12" s="24"/>
       <c r="H12" s="24"/>
     </row>
-    <row r="13" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="28"/>
+    <row r="13" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="27"/>
       <c r="C13" s="24"/>
       <c r="D13" s="24"/>
       <c r="E13" s="24"/>
@@ -3507,16 +3507,16 @@
       <c r="G13" s="24"/>
       <c r="H13" s="24"/>
     </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B15" s="4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C16" s="23" t="s">
+      <c r="C16" s="28" t="s">
         <v>7</v>
       </c>
       <c r="D16" s="24"/>
@@ -3525,11 +3525,11 @@
       <c r="G16" s="24"/>
       <c r="H16" s="24"/>
     </row>
-    <row r="17" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C17" s="23" t="s">
+      <c r="C17" s="28" t="s">
         <v>9</v>
       </c>
       <c r="D17" s="24"/>
@@ -3538,11 +3538,11 @@
       <c r="G17" s="24"/>
       <c r="H17" s="24"/>
     </row>
-    <row r="18" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C18" s="23" t="s">
+      <c r="C18" s="28" t="s">
         <v>11</v>
       </c>
       <c r="D18" s="24"/>
@@ -3551,11 +3551,11 @@
       <c r="G18" s="24"/>
       <c r="H18" s="24"/>
     </row>
-    <row r="19" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C19" s="23" t="s">
+      <c r="C19" s="28" t="s">
         <v>13</v>
       </c>
       <c r="D19" s="24"/>
@@ -3564,11 +3564,11 @@
       <c r="G19" s="24"/>
       <c r="H19" s="24"/>
     </row>
-    <row r="20" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C20" s="23" t="s">
+      <c r="C20" s="28" t="s">
         <v>15</v>
       </c>
       <c r="D20" s="24"/>
@@ -3577,11 +3577,11 @@
       <c r="G20" s="24"/>
       <c r="H20" s="24"/>
     </row>
-    <row r="21" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C21" s="23" t="s">
+      <c r="C21" s="28" t="s">
         <v>17</v>
       </c>
       <c r="D21" s="24"/>
@@ -3590,11 +3590,11 @@
       <c r="G21" s="24"/>
       <c r="H21" s="24"/>
     </row>
-    <row r="22" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C22" s="23" t="s">
+      <c r="C22" s="28" t="s">
         <v>19</v>
       </c>
       <c r="D22" s="24"/>
@@ -3603,11 +3603,11 @@
       <c r="G22" s="24"/>
       <c r="H22" s="24"/>
     </row>
-    <row r="23" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C23" s="23" t="s">
+      <c r="C23" s="28" t="s">
         <v>21</v>
       </c>
       <c r="D23" s="24"/>
@@ -3616,12 +3616,12 @@
       <c r="G23" s="24"/>
       <c r="H23" s="24"/>
     </row>
-    <row r="25" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B25" s="4" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="26" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B26" s="5" t="s">
         <v>23</v>
       </c>
@@ -3629,7 +3629,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B27" s="5" t="s">
         <v>24</v>
       </c>
@@ -3637,7 +3637,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="28" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B28" s="5" t="s">
         <v>25</v>
       </c>
@@ -3645,7 +3645,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B29" s="5" t="s">
         <v>26</v>
       </c>
@@ -3654,7 +3654,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="30" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B30" s="5" t="s">
         <v>27</v>
       </c>
@@ -3663,7 +3663,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="31" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B31" s="5" t="s">
         <v>28</v>
       </c>
@@ -3672,7 +3672,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="32" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B32" s="5" t="s">
         <v>29</v>
       </c>
@@ -3681,7 +3681,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="33" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B33" s="5" t="s">
         <v>30</v>
       </c>
@@ -3690,7 +3690,7 @@
         <v>0.53333333333333333</v>
       </c>
     </row>
-    <row r="34" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B34" s="5" t="s">
         <v>31</v>
       </c>
@@ -3699,12 +3699,12 @@
         <v>112</v>
       </c>
     </row>
-    <row r="36" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B36" s="4" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="37" spans="2:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="10" t="s">
         <v>33</v>
       </c>
@@ -3718,7 +3718,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="38" spans="2:8" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:8" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" s="11" t="s">
         <v>37</v>
       </c>
@@ -3734,7 +3734,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="39" spans="2:8" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:8" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="13" t="s">
         <v>39</v>
       </c>
@@ -3750,7 +3750,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="40" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B40" s="11" t="s">
         <v>41</v>
       </c>
@@ -3766,8 +3766,8 @@
         <v>8</v>
       </c>
     </row>
-    <row r="42" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B42" s="25" t="s">
+    <row r="42" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B42" s="23" t="s">
         <v>43</v>
       </c>
       <c r="C42" s="24"/>
@@ -3777,7 +3777,7 @@
       <c r="G42" s="24"/>
       <c r="H42" s="24"/>
     </row>
-    <row r="43" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B43" s="24"/>
       <c r="C43" s="24"/>
       <c r="D43" s="24"/>
@@ -3786,12 +3786,12 @@
       <c r="G43" s="24"/>
       <c r="H43" s="24"/>
     </row>
-    <row r="46" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B46" s="17" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="47" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B47" s="18" t="s">
         <v>45</v>
       </c>
@@ -3799,7 +3799,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="48" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B48" s="18" t="s">
         <v>47</v>
       </c>
@@ -3807,7 +3807,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="49" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B49" s="18" t="s">
         <v>49</v>
       </c>
@@ -3815,7 +3815,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="50" spans="2:3" ht="145.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:3" ht="145.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B50" s="18" t="s">
         <v>51</v>
       </c>
@@ -3823,7 +3823,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="51" spans="2:3" ht="52.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:3" ht="52.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B51" s="18" t="s">
         <v>53</v>
       </c>
@@ -3831,7 +3831,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="52" spans="2:3" ht="92.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:3" ht="92.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B52" s="18" t="s">
         <v>55</v>
       </c>
@@ -3839,7 +3839,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="53" spans="2:3" ht="118.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:3" ht="118.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B53" s="18" t="s">
         <v>57</v>
       </c>
@@ -3847,7 +3847,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="54" spans="2:3" ht="79.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:3" ht="79.150000000000006" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B54" s="18" t="s">
         <v>59</v>
       </c>
@@ -3855,7 +3855,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="55" spans="2:3" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:3" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B55" s="18" t="s">
         <v>61</v>
       </c>
@@ -3863,7 +3863,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="56" spans="2:3" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:3" ht="86.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B56" t="s">
         <v>63</v>
       </c>
@@ -3871,7 +3871,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="57" spans="2:3" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:3" ht="43.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B57" t="s">
         <v>65</v>
       </c>
@@ -3879,7 +3879,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="58" spans="2:3" ht="216" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:3" ht="216" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B58" t="s">
         <v>67</v>
       </c>
@@ -3920,25 +3920,25 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:P23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.77734375" customWidth="1"/>
-    <col min="2" max="2" width="9.77734375" customWidth="1"/>
-    <col min="3" max="3" width="40.77734375" customWidth="1"/>
-    <col min="4" max="4" width="24.77734375" customWidth="1"/>
-    <col min="5" max="5" width="32.77734375" customWidth="1"/>
-    <col min="6" max="7" width="13.77734375" customWidth="1"/>
-    <col min="8" max="8" width="6.77734375" customWidth="1"/>
-    <col min="9" max="9" width="8.77734375" customWidth="1"/>
-    <col min="10" max="10" width="10.77734375" customWidth="1"/>
-    <col min="11" max="11" width="15.77734375" customWidth="1"/>
-    <col min="12" max="12" width="10.77734375" customWidth="1"/>
-    <col min="13" max="14" width="13.77734375" customWidth="1"/>
-    <col min="15" max="15" width="15.77734375" customWidth="1"/>
-    <col min="16" max="16" width="28.77734375" customWidth="1"/>
+    <col min="1" max="1" width="10.7109375" customWidth="1"/>
+    <col min="2" max="2" width="9.7109375" customWidth="1"/>
+    <col min="3" max="3" width="40.7109375" customWidth="1"/>
+    <col min="4" max="4" width="24.7109375" customWidth="1"/>
+    <col min="5" max="5" width="32.7109375" customWidth="1"/>
+    <col min="6" max="7" width="13.7109375" customWidth="1"/>
+    <col min="8" max="8" width="6.7109375" customWidth="1"/>
+    <col min="9" max="9" width="8.7109375" customWidth="1"/>
+    <col min="10" max="10" width="10.7109375" customWidth="1"/>
+    <col min="11" max="11" width="15.7109375" customWidth="1"/>
+    <col min="12" max="12" width="10.7109375" customWidth="1"/>
+    <col min="13" max="14" width="13.7109375" customWidth="1"/>
+    <col min="15" max="15" width="15.7109375" customWidth="1"/>
+    <col min="16" max="16" width="28.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="24" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:16" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="29" t="s">
         <v>69</v>
       </c>
@@ -3958,7 +3958,7 @@
       <c r="O1" s="24"/>
       <c r="P1" s="24"/>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="30" t="s">
         <v>70</v>
       </c>
@@ -3978,7 +3978,7 @@
       <c r="O2" s="24"/>
       <c r="P2" s="24"/>
     </row>
-    <row r="5" spans="1:16" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>71</v>
       </c>
@@ -4028,7 +4028,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" ht="110.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
         <v>86</v>
       </c>
@@ -4079,7 +4079,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" ht="110.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
         <v>96</v>
       </c>
@@ -4130,7 +4130,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="96.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" ht="96.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
         <v>102</v>
       </c>
@@ -4181,7 +4181,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" ht="82.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
         <v>110</v>
       </c>
@@ -4232,7 +4232,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" ht="110.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
         <v>117</v>
       </c>
@@ -4283,7 +4283,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="96.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" ht="96.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
         <v>108</v>
       </c>
@@ -4334,7 +4334,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16" ht="55.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
         <v>127</v>
       </c>
@@ -4385,7 +4385,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="96.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16" ht="96.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
         <v>132</v>
       </c>
@@ -4436,7 +4436,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="14" spans="1:16" ht="96.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:16" ht="96.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
         <v>125</v>
       </c>
@@ -4487,7 +4487,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="15" spans="1:16" ht="69" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:16" ht="69" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
         <v>142</v>
       </c>
@@ -4538,7 +4538,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="69" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:16" ht="69" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
         <v>147</v>
       </c>
@@ -4589,7 +4589,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="17" spans="1:16" ht="69" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:16" ht="69" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
         <v>152</v>
       </c>
@@ -4640,7 +4640,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="18" spans="1:16" ht="124.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:16" ht="124.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
         <v>157</v>
       </c>
@@ -4691,7 +4691,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="19" spans="1:16" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:16" ht="55.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
         <v>165</v>
       </c>
@@ -4742,7 +4742,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="20" spans="1:16" ht="69" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:16" ht="69" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
         <v>171</v>
       </c>
@@ -4793,7 +4793,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="21" spans="1:16" ht="124.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:16" ht="124.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
         <v>176</v>
       </c>
@@ -4844,7 +4844,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="22" spans="1:16" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:16" ht="82.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
         <v>169</v>
       </c>
@@ -4895,7 +4895,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" s="15"/>
       <c r="B23" s="15"/>
       <c r="C23" s="16" t="s">
@@ -4969,21 +4969,21 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:J256"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.77734375" customWidth="1"/>
-    <col min="2" max="2" width="13.77734375" customWidth="1"/>
-    <col min="3" max="3" width="38.77734375" customWidth="1"/>
-    <col min="4" max="4" width="46.77734375" customWidth="1"/>
-    <col min="5" max="5" width="15.77734375" customWidth="1"/>
-    <col min="6" max="6" width="10.77734375" customWidth="1"/>
-    <col min="7" max="7" width="16.77734375" customWidth="1"/>
-    <col min="8" max="8" width="13.77734375" customWidth="1"/>
-    <col min="9" max="9" width="11.77734375" customWidth="1"/>
-    <col min="10" max="10" width="28.77734375" customWidth="1"/>
+    <col min="1" max="1" width="10.7109375" customWidth="1"/>
+    <col min="2" max="2" width="13.7109375" customWidth="1"/>
+    <col min="3" max="3" width="38.7109375" customWidth="1"/>
+    <col min="4" max="4" width="46.7109375" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" customWidth="1"/>
+    <col min="6" max="6" width="10.7109375" customWidth="1"/>
+    <col min="7" max="7" width="16.7109375" customWidth="1"/>
+    <col min="8" max="8" width="13.7109375" customWidth="1"/>
+    <col min="9" max="9" width="11.7109375" customWidth="1"/>
+    <col min="10" max="10" width="28.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="29" t="s">
         <v>186</v>
       </c>
@@ -4997,7 +4997,7 @@
       <c r="I1" s="24"/>
       <c r="J1" s="24"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="30" t="s">
         <v>187</v>
       </c>
@@ -5011,7 +5011,7 @@
       <c r="I2" s="24"/>
       <c r="J2" s="24"/>
     </row>
-    <row r="5" spans="1:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>188</v>
       </c>
@@ -5043,7 +5043,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
         <v>194</v>
       </c>
@@ -5071,7 +5071,7 @@
       <c r="I6" s="11"/>
       <c r="J6" s="20"/>
     </row>
-    <row r="7" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
         <v>198</v>
       </c>
@@ -5099,7 +5099,7 @@
       <c r="I7" s="11"/>
       <c r="J7" s="20"/>
     </row>
-    <row r="8" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
         <v>200</v>
       </c>
@@ -5127,7 +5127,7 @@
       <c r="I8" s="11"/>
       <c r="J8" s="20"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
         <v>202</v>
       </c>
@@ -5155,7 +5155,7 @@
       <c r="I9" s="11"/>
       <c r="J9" s="20"/>
     </row>
-    <row r="10" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
         <v>204</v>
       </c>
@@ -5183,7 +5183,7 @@
       <c r="I10" s="11"/>
       <c r="J10" s="20"/>
     </row>
-    <row r="11" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
         <v>206</v>
       </c>
@@ -5215,7 +5215,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
         <v>210</v>
       </c>
@@ -5247,7 +5247,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
         <v>213</v>
       </c>
@@ -5275,7 +5275,7 @@
       <c r="I13" s="11"/>
       <c r="J13" s="20"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
         <v>215</v>
       </c>
@@ -5303,7 +5303,7 @@
       <c r="I14" s="11"/>
       <c r="J14" s="20"/>
     </row>
-    <row r="15" spans="1:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" ht="55.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
         <v>219</v>
       </c>
@@ -5331,7 +5331,7 @@
       <c r="I15" s="11"/>
       <c r="J15" s="20"/>
     </row>
-    <row r="16" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
         <v>222</v>
       </c>
@@ -5359,7 +5359,7 @@
       <c r="I16" s="11"/>
       <c r="J16" s="20"/>
     </row>
-    <row r="17" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
         <v>225</v>
       </c>
@@ -5387,7 +5387,7 @@
       <c r="I17" s="11"/>
       <c r="J17" s="20"/>
     </row>
-    <row r="18" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
         <v>228</v>
       </c>
@@ -5407,7 +5407,7 @@
         <v>0.75</v>
       </c>
       <c r="G18" s="12" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="H18" s="11" t="s">
         <v>218</v>
@@ -5417,7 +5417,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
         <v>231</v>
       </c>
@@ -5445,7 +5445,7 @@
       <c r="I19" s="11"/>
       <c r="J19" s="20"/>
     </row>
-    <row r="20" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
         <v>233</v>
       </c>
@@ -5473,7 +5473,7 @@
       <c r="I20" s="11"/>
       <c r="J20" s="20"/>
     </row>
-    <row r="21" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
         <v>235</v>
       </c>
@@ -5501,7 +5501,7 @@
       <c r="I21" s="11"/>
       <c r="J21" s="20"/>
     </row>
-    <row r="22" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
         <v>237</v>
       </c>
@@ -5529,7 +5529,7 @@
       <c r="I22" s="11"/>
       <c r="J22" s="20"/>
     </row>
-    <row r="23" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
         <v>239</v>
       </c>
@@ -5561,7 +5561,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
         <v>242</v>
       </c>
@@ -5593,7 +5593,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
         <v>245</v>
       </c>
@@ -5621,7 +5621,7 @@
       <c r="I25" s="11"/>
       <c r="J25" s="20"/>
     </row>
-    <row r="26" spans="1:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:10" ht="55.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
         <v>247</v>
       </c>
@@ -5649,7 +5649,7 @@
       <c r="I26" s="11"/>
       <c r="J26" s="20"/>
     </row>
-    <row r="27" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="11" t="s">
         <v>248</v>
       </c>
@@ -5677,7 +5677,7 @@
       <c r="I27" s="11"/>
       <c r="J27" s="20"/>
     </row>
-    <row r="28" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="11" t="s">
         <v>249</v>
       </c>
@@ -5705,7 +5705,7 @@
       <c r="I28" s="11"/>
       <c r="J28" s="20"/>
     </row>
-    <row r="29" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
         <v>250</v>
       </c>
@@ -5733,7 +5733,7 @@
       <c r="I29" s="11"/>
       <c r="J29" s="20"/>
     </row>
-    <row r="30" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="11" t="s">
         <v>251</v>
       </c>
@@ -5763,7 +5763,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="11" t="s">
         <v>253</v>
       </c>
@@ -5793,7 +5793,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="11" t="s">
         <v>255</v>
       </c>
@@ -5823,7 +5823,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="33" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="11" t="s">
         <v>257</v>
       </c>
@@ -5853,7 +5853,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="11" t="s">
         <v>259</v>
       </c>
@@ -5883,7 +5883,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="35" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="11" t="s">
         <v>261</v>
       </c>
@@ -5911,7 +5911,7 @@
       <c r="I35" s="11"/>
       <c r="J35" s="20"/>
     </row>
-    <row r="36" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="11" t="s">
         <v>263</v>
       </c>
@@ -5939,7 +5939,7 @@
       <c r="I36" s="11"/>
       <c r="J36" s="20"/>
     </row>
-    <row r="37" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="11" t="s">
         <v>265</v>
       </c>
@@ -5967,7 +5967,7 @@
       <c r="I37" s="11"/>
       <c r="J37" s="20"/>
     </row>
-    <row r="38" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="11" t="s">
         <v>267</v>
       </c>
@@ -5995,7 +5995,7 @@
       <c r="I38" s="11"/>
       <c r="J38" s="20"/>
     </row>
-    <row r="39" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="11" t="s">
         <v>269</v>
       </c>
@@ -6023,7 +6023,7 @@
       <c r="I39" s="11"/>
       <c r="J39" s="20"/>
     </row>
-    <row r="40" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="11" t="s">
         <v>271</v>
       </c>
@@ -6051,7 +6051,7 @@
       <c r="I40" s="11"/>
       <c r="J40" s="20"/>
     </row>
-    <row r="41" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="11" t="s">
         <v>273</v>
       </c>
@@ -6083,7 +6083,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="42" spans="1:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:10" ht="55.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="11" t="s">
         <v>277</v>
       </c>
@@ -6115,7 +6115,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="43" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="11" t="s">
         <v>280</v>
       </c>
@@ -6147,7 +6147,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="44" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="11" t="s">
         <v>283</v>
       </c>
@@ -6179,7 +6179,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="45" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="11" t="s">
         <v>286</v>
       </c>
@@ -6207,7 +6207,7 @@
       <c r="I45" s="11"/>
       <c r="J45" s="20"/>
     </row>
-    <row r="46" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="11" t="s">
         <v>288</v>
       </c>
@@ -6235,7 +6235,7 @@
       <c r="I46" s="11"/>
       <c r="J46" s="20"/>
     </row>
-    <row r="47" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="11" t="s">
         <v>290</v>
       </c>
@@ -6263,7 +6263,7 @@
       <c r="I47" s="11"/>
       <c r="J47" s="20"/>
     </row>
-    <row r="48" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="11" t="s">
         <v>292</v>
       </c>
@@ -6291,7 +6291,7 @@
       <c r="I48" s="11"/>
       <c r="J48" s="20"/>
     </row>
-    <row r="49" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="11" t="s">
         <v>293</v>
       </c>
@@ -6319,7 +6319,7 @@
       <c r="I49" s="11"/>
       <c r="J49" s="20"/>
     </row>
-    <row r="50" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="11" t="s">
         <v>294</v>
       </c>
@@ -6347,7 +6347,7 @@
       <c r="I50" s="11"/>
       <c r="J50" s="20"/>
     </row>
-    <row r="51" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="11" t="s">
         <v>295</v>
       </c>
@@ -6375,7 +6375,7 @@
       <c r="I51" s="11"/>
       <c r="J51" s="20"/>
     </row>
-    <row r="52" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="11" t="s">
         <v>298</v>
       </c>
@@ -6403,7 +6403,7 @@
       <c r="I52" s="11"/>
       <c r="J52" s="20"/>
     </row>
-    <row r="53" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="11" t="s">
         <v>299</v>
       </c>
@@ -6431,7 +6431,7 @@
       <c r="I53" s="11"/>
       <c r="J53" s="20"/>
     </row>
-    <row r="54" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="11" t="s">
         <v>301</v>
       </c>
@@ -6459,7 +6459,7 @@
       <c r="I54" s="11"/>
       <c r="J54" s="20"/>
     </row>
-    <row r="55" spans="1:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:10" ht="55.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="11" t="s">
         <v>302</v>
       </c>
@@ -6487,7 +6487,7 @@
       <c r="I55" s="11"/>
       <c r="J55" s="20"/>
     </row>
-    <row r="56" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="11" t="s">
         <v>304</v>
       </c>
@@ -6515,7 +6515,7 @@
       <c r="I56" s="11"/>
       <c r="J56" s="20"/>
     </row>
-    <row r="57" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="11" t="s">
         <v>305</v>
       </c>
@@ -6547,7 +6547,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="58" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="11" t="s">
         <v>308</v>
       </c>
@@ -6579,7 +6579,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="59" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="11" t="s">
         <v>310</v>
       </c>
@@ -6607,7 +6607,7 @@
       <c r="I59" s="11"/>
       <c r="J59" s="20"/>
     </row>
-    <row r="60" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="11" t="s">
         <v>312</v>
       </c>
@@ -6635,7 +6635,7 @@
       <c r="I60" s="11"/>
       <c r="J60" s="20"/>
     </row>
-    <row r="61" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="11" t="s">
         <v>313</v>
       </c>
@@ -6663,7 +6663,7 @@
       <c r="I61" s="11"/>
       <c r="J61" s="20"/>
     </row>
-    <row r="62" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="11" t="s">
         <v>314</v>
       </c>
@@ -6691,7 +6691,7 @@
       <c r="I62" s="11"/>
       <c r="J62" s="20"/>
     </row>
-    <row r="63" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="11" t="s">
         <v>315</v>
       </c>
@@ -6719,7 +6719,7 @@
       <c r="I63" s="11"/>
       <c r="J63" s="20"/>
     </row>
-    <row r="64" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="11" t="s">
         <v>316</v>
       </c>
@@ -6747,7 +6747,7 @@
       <c r="I64" s="11"/>
       <c r="J64" s="20"/>
     </row>
-    <row r="65" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="11" t="s">
         <v>318</v>
       </c>
@@ -6775,7 +6775,7 @@
       <c r="I65" s="11"/>
       <c r="J65" s="20"/>
     </row>
-    <row r="66" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="11" t="s">
         <v>320</v>
       </c>
@@ -6803,7 +6803,7 @@
       <c r="I66" s="11"/>
       <c r="J66" s="20"/>
     </row>
-    <row r="67" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="11" t="s">
         <v>322</v>
       </c>
@@ -6831,7 +6831,7 @@
       <c r="I67" s="11"/>
       <c r="J67" s="20"/>
     </row>
-    <row r="68" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="11" t="s">
         <v>324</v>
       </c>
@@ -6859,7 +6859,7 @@
       <c r="I68" s="11"/>
       <c r="J68" s="20"/>
     </row>
-    <row r="69" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="11" t="s">
         <v>326</v>
       </c>
@@ -6887,7 +6887,7 @@
       <c r="I69" s="11"/>
       <c r="J69" s="20"/>
     </row>
-    <row r="70" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="11" t="s">
         <v>328</v>
       </c>
@@ -6919,7 +6919,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="71" spans="1:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:10" ht="55.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="11" t="s">
         <v>331</v>
       </c>
@@ -6951,7 +6951,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="72" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="11" t="s">
         <v>334</v>
       </c>
@@ -6983,7 +6983,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="73" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="11" t="s">
         <v>337</v>
       </c>
@@ -7015,7 +7015,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="74" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="11" t="s">
         <v>340</v>
       </c>
@@ -7043,7 +7043,7 @@
       <c r="I74" s="11"/>
       <c r="J74" s="20"/>
     </row>
-    <row r="75" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="11" t="s">
         <v>342</v>
       </c>
@@ -7071,7 +7071,7 @@
       <c r="I75" s="11"/>
       <c r="J75" s="20"/>
     </row>
-    <row r="76" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="11" t="s">
         <v>344</v>
       </c>
@@ -7099,7 +7099,7 @@
       <c r="I76" s="11"/>
       <c r="J76" s="20"/>
     </row>
-    <row r="77" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="11" t="s">
         <v>345</v>
       </c>
@@ -7127,7 +7127,7 @@
       <c r="I77" s="11"/>
       <c r="J77" s="20"/>
     </row>
-    <row r="78" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="11" t="s">
         <v>346</v>
       </c>
@@ -7155,7 +7155,7 @@
       <c r="I78" s="11"/>
       <c r="J78" s="20"/>
     </row>
-    <row r="79" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="11" t="s">
         <v>347</v>
       </c>
@@ -7183,7 +7183,7 @@
       <c r="I79" s="11"/>
       <c r="J79" s="20"/>
     </row>
-    <row r="80" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="11" t="s">
         <v>348</v>
       </c>
@@ -7211,7 +7211,7 @@
       <c r="I80" s="11"/>
       <c r="J80" s="20"/>
     </row>
-    <row r="81" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="11" t="s">
         <v>349</v>
       </c>
@@ -7239,7 +7239,7 @@
       <c r="I81" s="11"/>
       <c r="J81" s="20"/>
     </row>
-    <row r="82" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="11" t="s">
         <v>351</v>
       </c>
@@ -7267,7 +7267,7 @@
       <c r="I82" s="11"/>
       <c r="J82" s="20"/>
     </row>
-    <row r="83" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="11" t="s">
         <v>353</v>
       </c>
@@ -7295,7 +7295,7 @@
       <c r="I83" s="11"/>
       <c r="J83" s="20"/>
     </row>
-    <row r="84" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="11" t="s">
         <v>355</v>
       </c>
@@ -7323,7 +7323,7 @@
       <c r="I84" s="11"/>
       <c r="J84" s="20"/>
     </row>
-    <row r="85" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="11" t="s">
         <v>357</v>
       </c>
@@ -7351,7 +7351,7 @@
       <c r="I85" s="11"/>
       <c r="J85" s="20"/>
     </row>
-    <row r="86" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="11" t="s">
         <v>359</v>
       </c>
@@ -7379,7 +7379,7 @@
       <c r="I86" s="11"/>
       <c r="J86" s="20"/>
     </row>
-    <row r="87" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="11" t="s">
         <v>361</v>
       </c>
@@ -7411,7 +7411,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="88" spans="1:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:10" ht="55.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="11" t="s">
         <v>364</v>
       </c>
@@ -7443,7 +7443,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="89" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="11" t="s">
         <v>367</v>
       </c>
@@ -7475,7 +7475,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="90" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="11" t="s">
         <v>370</v>
       </c>
@@ -7507,7 +7507,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="91" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="11" t="s">
         <v>373</v>
       </c>
@@ -7535,7 +7535,7 @@
       <c r="I91" s="11"/>
       <c r="J91" s="20"/>
     </row>
-    <row r="92" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="11" t="s">
         <v>375</v>
       </c>
@@ -7563,7 +7563,7 @@
       <c r="I92" s="11"/>
       <c r="J92" s="20"/>
     </row>
-    <row r="93" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="11" t="s">
         <v>377</v>
       </c>
@@ -7591,7 +7591,7 @@
       <c r="I93" s="11"/>
       <c r="J93" s="20"/>
     </row>
-    <row r="94" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="11" t="s">
         <v>378</v>
       </c>
@@ -7619,7 +7619,7 @@
       <c r="I94" s="11"/>
       <c r="J94" s="20"/>
     </row>
-    <row r="95" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="11" t="s">
         <v>379</v>
       </c>
@@ -7647,7 +7647,7 @@
       <c r="I95" s="11"/>
       <c r="J95" s="20"/>
     </row>
-    <row r="96" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="11" t="s">
         <v>380</v>
       </c>
@@ -7675,7 +7675,7 @@
       <c r="I96" s="11"/>
       <c r="J96" s="20"/>
     </row>
-    <row r="97" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="11" t="s">
         <v>381</v>
       </c>
@@ -7703,7 +7703,7 @@
       <c r="I97" s="11"/>
       <c r="J97" s="20"/>
     </row>
-    <row r="98" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="11" t="s">
         <v>383</v>
       </c>
@@ -7731,7 +7731,7 @@
       <c r="I98" s="11"/>
       <c r="J98" s="20"/>
     </row>
-    <row r="99" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="11" t="s">
         <v>385</v>
       </c>
@@ -7759,7 +7759,7 @@
       <c r="I99" s="11"/>
       <c r="J99" s="20"/>
     </row>
-    <row r="100" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="11" t="s">
         <v>387</v>
       </c>
@@ -7787,7 +7787,7 @@
       <c r="I100" s="11"/>
       <c r="J100" s="20"/>
     </row>
-    <row r="101" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="11" t="s">
         <v>389</v>
       </c>
@@ -7815,7 +7815,7 @@
       <c r="I101" s="11"/>
       <c r="J101" s="20"/>
     </row>
-    <row r="102" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="11" t="s">
         <v>391</v>
       </c>
@@ -7843,7 +7843,7 @@
       <c r="I102" s="11"/>
       <c r="J102" s="20"/>
     </row>
-    <row r="103" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="11" t="s">
         <v>393</v>
       </c>
@@ -7875,7 +7875,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="104" spans="1:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:10" ht="55.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="11" t="s">
         <v>396</v>
       </c>
@@ -7907,7 +7907,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="105" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="11" t="s">
         <v>399</v>
       </c>
@@ -7939,7 +7939,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="106" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="11" t="s">
         <v>402</v>
       </c>
@@ -7971,7 +7971,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="107" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="11" t="s">
         <v>405</v>
       </c>
@@ -7999,7 +7999,7 @@
       <c r="I107" s="11"/>
       <c r="J107" s="20"/>
     </row>
-    <row r="108" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="11" t="s">
         <v>407</v>
       </c>
@@ -8027,7 +8027,7 @@
       <c r="I108" s="11"/>
       <c r="J108" s="20"/>
     </row>
-    <row r="109" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109" s="11" t="s">
         <v>409</v>
       </c>
@@ -8055,7 +8055,7 @@
       <c r="I109" s="11"/>
       <c r="J109" s="20"/>
     </row>
-    <row r="110" spans="1:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:10" ht="55.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="11" t="s">
         <v>410</v>
       </c>
@@ -8083,7 +8083,7 @@
       <c r="I110" s="11"/>
       <c r="J110" s="20"/>
     </row>
-    <row r="111" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="11" t="s">
         <v>411</v>
       </c>
@@ -8111,7 +8111,7 @@
       <c r="I111" s="11"/>
       <c r="J111" s="20"/>
     </row>
-    <row r="112" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="11" t="s">
         <v>412</v>
       </c>
@@ -8139,7 +8139,7 @@
       <c r="I112" s="11"/>
       <c r="J112" s="20"/>
     </row>
-    <row r="113" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113" s="11" t="s">
         <v>413</v>
       </c>
@@ -8167,7 +8167,7 @@
       <c r="I113" s="11"/>
       <c r="J113" s="20"/>
     </row>
-    <row r="114" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A114" s="11" t="s">
         <v>414</v>
       </c>
@@ -8195,7 +8195,7 @@
       <c r="I114" s="11"/>
       <c r="J114" s="20"/>
     </row>
-    <row r="115" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A115" s="11" t="s">
         <v>415</v>
       </c>
@@ -8223,7 +8223,7 @@
       <c r="I115" s="11"/>
       <c r="J115" s="20"/>
     </row>
-    <row r="116" spans="1:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:10" ht="55.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="11" t="s">
         <v>416</v>
       </c>
@@ -8251,7 +8251,7 @@
       <c r="I116" s="11"/>
       <c r="J116" s="20"/>
     </row>
-    <row r="117" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="11" t="s">
         <v>417</v>
       </c>
@@ -8279,7 +8279,7 @@
       <c r="I117" s="11"/>
       <c r="J117" s="20"/>
     </row>
-    <row r="118" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A118" s="11" t="s">
         <v>418</v>
       </c>
@@ -8311,7 +8311,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="119" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119" s="11" t="s">
         <v>420</v>
       </c>
@@ -8343,7 +8343,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="120" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="11" t="s">
         <v>422</v>
       </c>
@@ -8371,7 +8371,7 @@
       <c r="I120" s="11"/>
       <c r="J120" s="20"/>
     </row>
-    <row r="121" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A121" s="11" t="s">
         <v>423</v>
       </c>
@@ -8399,7 +8399,7 @@
       <c r="I121" s="11"/>
       <c r="J121" s="20"/>
     </row>
-    <row r="122" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="11" t="s">
         <v>424</v>
       </c>
@@ -8427,7 +8427,7 @@
       <c r="I122" s="11"/>
       <c r="J122" s="20"/>
     </row>
-    <row r="123" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A123" s="11" t="s">
         <v>425</v>
       </c>
@@ -8455,7 +8455,7 @@
       <c r="I123" s="11"/>
       <c r="J123" s="20"/>
     </row>
-    <row r="124" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A124" s="11" t="s">
         <v>426</v>
       </c>
@@ -8483,7 +8483,7 @@
       <c r="I124" s="11"/>
       <c r="J124" s="20"/>
     </row>
-    <row r="125" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125" s="11" t="s">
         <v>427</v>
       </c>
@@ -8511,7 +8511,7 @@
       <c r="I125" s="11"/>
       <c r="J125" s="20"/>
     </row>
-    <row r="126" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A126" s="11" t="s">
         <v>429</v>
       </c>
@@ -8539,7 +8539,7 @@
       <c r="I126" s="11"/>
       <c r="J126" s="20"/>
     </row>
-    <row r="127" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A127" s="11" t="s">
         <v>431</v>
       </c>
@@ -8567,7 +8567,7 @@
       <c r="I127" s="11"/>
       <c r="J127" s="20"/>
     </row>
-    <row r="128" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A128" s="11" t="s">
         <v>433</v>
       </c>
@@ -8595,7 +8595,7 @@
       <c r="I128" s="11"/>
       <c r="J128" s="20"/>
     </row>
-    <row r="129" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129" s="11" t="s">
         <v>435</v>
       </c>
@@ -8623,7 +8623,7 @@
       <c r="I129" s="11"/>
       <c r="J129" s="20"/>
     </row>
-    <row r="130" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130" s="11" t="s">
         <v>437</v>
       </c>
@@ -8651,7 +8651,7 @@
       <c r="I130" s="11"/>
       <c r="J130" s="20"/>
     </row>
-    <row r="131" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="11" t="s">
         <v>439</v>
       </c>
@@ -8683,7 +8683,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="132" spans="1:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:10" ht="55.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A132" s="11" t="s">
         <v>442</v>
       </c>
@@ -8715,7 +8715,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="133" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A133" s="11" t="s">
         <v>445</v>
       </c>
@@ -8747,7 +8747,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="134" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A134" s="11" t="s">
         <v>448</v>
       </c>
@@ -8779,7 +8779,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="135" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A135" s="11" t="s">
         <v>451</v>
       </c>
@@ -8807,7 +8807,7 @@
       <c r="I135" s="11"/>
       <c r="J135" s="20"/>
     </row>
-    <row r="136" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A136" s="11" t="s">
         <v>453</v>
       </c>
@@ -8835,7 +8835,7 @@
       <c r="I136" s="11"/>
       <c r="J136" s="20"/>
     </row>
-    <row r="137" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A137" s="11" t="s">
         <v>455</v>
       </c>
@@ -8863,7 +8863,7 @@
       <c r="I137" s="11"/>
       <c r="J137" s="20"/>
     </row>
-    <row r="138" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A138" s="11" t="s">
         <v>456</v>
       </c>
@@ -8891,7 +8891,7 @@
       <c r="I138" s="11"/>
       <c r="J138" s="20"/>
     </row>
-    <row r="139" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A139" s="11" t="s">
         <v>457</v>
       </c>
@@ -8919,7 +8919,7 @@
       <c r="I139" s="11"/>
       <c r="J139" s="20"/>
     </row>
-    <row r="140" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A140" s="11" t="s">
         <v>458</v>
       </c>
@@ -8947,7 +8947,7 @@
       <c r="I140" s="11"/>
       <c r="J140" s="20"/>
     </row>
-    <row r="141" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A141" s="11" t="s">
         <v>459</v>
       </c>
@@ -8975,7 +8975,7 @@
       <c r="I141" s="11"/>
       <c r="J141" s="20"/>
     </row>
-    <row r="142" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A142" s="11" t="s">
         <v>461</v>
       </c>
@@ -9003,7 +9003,7 @@
       <c r="I142" s="11"/>
       <c r="J142" s="20"/>
     </row>
-    <row r="143" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A143" s="11" t="s">
         <v>463</v>
       </c>
@@ -9031,7 +9031,7 @@
       <c r="I143" s="11"/>
       <c r="J143" s="20"/>
     </row>
-    <row r="144" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A144" s="11" t="s">
         <v>465</v>
       </c>
@@ -9059,7 +9059,7 @@
       <c r="I144" s="11"/>
       <c r="J144" s="20"/>
     </row>
-    <row r="145" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A145" s="11" t="s">
         <v>467</v>
       </c>
@@ -9087,7 +9087,7 @@
       <c r="I145" s="11"/>
       <c r="J145" s="20"/>
     </row>
-    <row r="146" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A146" s="11" t="s">
         <v>469</v>
       </c>
@@ -9115,7 +9115,7 @@
       <c r="I146" s="11"/>
       <c r="J146" s="20"/>
     </row>
-    <row r="147" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A147" s="11" t="s">
         <v>471</v>
       </c>
@@ -9147,7 +9147,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="148" spans="1:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:10" ht="55.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A148" s="11" t="s">
         <v>474</v>
       </c>
@@ -9179,7 +9179,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="149" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A149" s="11" t="s">
         <v>477</v>
       </c>
@@ -9211,7 +9211,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="150" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A150" s="11" t="s">
         <v>480</v>
       </c>
@@ -9243,7 +9243,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="151" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A151" s="11" t="s">
         <v>483</v>
       </c>
@@ -9271,7 +9271,7 @@
       <c r="I151" s="11"/>
       <c r="J151" s="20"/>
     </row>
-    <row r="152" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A152" s="11" t="s">
         <v>485</v>
       </c>
@@ -9299,7 +9299,7 @@
       <c r="I152" s="11"/>
       <c r="J152" s="20"/>
     </row>
-    <row r="153" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A153" s="11" t="s">
         <v>487</v>
       </c>
@@ -9327,7 +9327,7 @@
       <c r="I153" s="11"/>
       <c r="J153" s="20"/>
     </row>
-    <row r="154" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A154" s="11" t="s">
         <v>488</v>
       </c>
@@ -9355,7 +9355,7 @@
       <c r="I154" s="11"/>
       <c r="J154" s="20"/>
     </row>
-    <row r="155" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A155" s="11" t="s">
         <v>489</v>
       </c>
@@ -9383,7 +9383,7 @@
       <c r="I155" s="11"/>
       <c r="J155" s="20"/>
     </row>
-    <row r="156" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A156" s="11" t="s">
         <v>490</v>
       </c>
@@ -9411,7 +9411,7 @@
       <c r="I156" s="11"/>
       <c r="J156" s="20"/>
     </row>
-    <row r="157" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A157" s="11" t="s">
         <v>491</v>
       </c>
@@ -9439,7 +9439,7 @@
       <c r="I157" s="11"/>
       <c r="J157" s="20"/>
     </row>
-    <row r="158" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A158" s="11" t="s">
         <v>493</v>
       </c>
@@ -9467,7 +9467,7 @@
       <c r="I158" s="11"/>
       <c r="J158" s="20"/>
     </row>
-    <row r="159" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A159" s="11" t="s">
         <v>495</v>
       </c>
@@ -9495,7 +9495,7 @@
       <c r="I159" s="11"/>
       <c r="J159" s="20"/>
     </row>
-    <row r="160" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A160" s="11" t="s">
         <v>497</v>
       </c>
@@ -9523,7 +9523,7 @@
       <c r="I160" s="11"/>
       <c r="J160" s="20"/>
     </row>
-    <row r="161" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A161" s="11" t="s">
         <v>499</v>
       </c>
@@ -9551,7 +9551,7 @@
       <c r="I161" s="11"/>
       <c r="J161" s="20"/>
     </row>
-    <row r="162" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A162" s="11" t="s">
         <v>501</v>
       </c>
@@ -9579,7 +9579,7 @@
       <c r="I162" s="11"/>
       <c r="J162" s="20"/>
     </row>
-    <row r="163" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A163" s="11" t="s">
         <v>503</v>
       </c>
@@ -9611,7 +9611,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="164" spans="1:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:10" ht="55.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A164" s="11" t="s">
         <v>506</v>
       </c>
@@ -9643,7 +9643,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="165" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A165" s="11" t="s">
         <v>509</v>
       </c>
@@ -9675,7 +9675,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="166" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A166" s="11" t="s">
         <v>512</v>
       </c>
@@ -9707,7 +9707,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="167" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A167" s="11" t="s">
         <v>515</v>
       </c>
@@ -9735,7 +9735,7 @@
       <c r="I167" s="11"/>
       <c r="J167" s="20"/>
     </row>
-    <row r="168" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A168" s="11" t="s">
         <v>517</v>
       </c>
@@ -9763,7 +9763,7 @@
       <c r="I168" s="11"/>
       <c r="J168" s="20"/>
     </row>
-    <row r="169" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A169" s="11" t="s">
         <v>519</v>
       </c>
@@ -9791,7 +9791,7 @@
       <c r="I169" s="11"/>
       <c r="J169" s="20"/>
     </row>
-    <row r="170" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A170" s="11" t="s">
         <v>520</v>
       </c>
@@ -9819,7 +9819,7 @@
       <c r="I170" s="11"/>
       <c r="J170" s="20"/>
     </row>
-    <row r="171" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A171" s="11" t="s">
         <v>521</v>
       </c>
@@ -9847,7 +9847,7 @@
       <c r="I171" s="11"/>
       <c r="J171" s="20"/>
     </row>
-    <row r="172" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A172" s="11" t="s">
         <v>522</v>
       </c>
@@ -9875,7 +9875,7 @@
       <c r="I172" s="11"/>
       <c r="J172" s="20"/>
     </row>
-    <row r="173" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A173" s="11" t="s">
         <v>523</v>
       </c>
@@ -9903,7 +9903,7 @@
       <c r="I173" s="11"/>
       <c r="J173" s="20"/>
     </row>
-    <row r="174" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A174" s="11" t="s">
         <v>525</v>
       </c>
@@ -9931,7 +9931,7 @@
       <c r="I174" s="11"/>
       <c r="J174" s="20"/>
     </row>
-    <row r="175" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A175" s="11" t="s">
         <v>527</v>
       </c>
@@ -9959,7 +9959,7 @@
       <c r="I175" s="11"/>
       <c r="J175" s="20"/>
     </row>
-    <row r="176" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A176" s="11" t="s">
         <v>529</v>
       </c>
@@ -9987,7 +9987,7 @@
       <c r="I176" s="11"/>
       <c r="J176" s="20"/>
     </row>
-    <row r="177" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A177" s="11" t="s">
         <v>531</v>
       </c>
@@ -10015,7 +10015,7 @@
       <c r="I177" s="11"/>
       <c r="J177" s="20"/>
     </row>
-    <row r="178" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A178" s="11" t="s">
         <v>533</v>
       </c>
@@ -10043,7 +10043,7 @@
       <c r="I178" s="11"/>
       <c r="J178" s="20"/>
     </row>
-    <row r="179" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A179" s="11" t="s">
         <v>535</v>
       </c>
@@ -10075,7 +10075,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="180" spans="1:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:10" ht="55.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A180" s="11" t="s">
         <v>538</v>
       </c>
@@ -10107,7 +10107,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="181" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A181" s="11" t="s">
         <v>541</v>
       </c>
@@ -10139,7 +10139,7 @@
         <v>543</v>
       </c>
     </row>
-    <row r="182" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A182" s="11" t="s">
         <v>544</v>
       </c>
@@ -10171,7 +10171,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="183" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A183" s="11" t="s">
         <v>547</v>
       </c>
@@ -10199,7 +10199,7 @@
       <c r="I183" s="11"/>
       <c r="J183" s="20"/>
     </row>
-    <row r="184" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A184" s="11" t="s">
         <v>549</v>
       </c>
@@ -10227,7 +10227,7 @@
       <c r="I184" s="11"/>
       <c r="J184" s="20"/>
     </row>
-    <row r="185" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A185" s="11" t="s">
         <v>551</v>
       </c>
@@ -10255,7 +10255,7 @@
       <c r="I185" s="11"/>
       <c r="J185" s="20"/>
     </row>
-    <row r="186" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A186" s="11" t="s">
         <v>552</v>
       </c>
@@ -10283,7 +10283,7 @@
       <c r="I186" s="11"/>
       <c r="J186" s="20"/>
     </row>
-    <row r="187" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A187" s="11" t="s">
         <v>553</v>
       </c>
@@ -10311,7 +10311,7 @@
       <c r="I187" s="11"/>
       <c r="J187" s="20"/>
     </row>
-    <row r="188" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A188" s="11" t="s">
         <v>554</v>
       </c>
@@ -10339,7 +10339,7 @@
       <c r="I188" s="11"/>
       <c r="J188" s="20"/>
     </row>
-    <row r="189" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A189" s="11" t="s">
         <v>555</v>
       </c>
@@ -10367,7 +10367,7 @@
       <c r="I189" s="11"/>
       <c r="J189" s="20"/>
     </row>
-    <row r="190" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A190" s="11" t="s">
         <v>557</v>
       </c>
@@ -10395,7 +10395,7 @@
       <c r="I190" s="11"/>
       <c r="J190" s="20"/>
     </row>
-    <row r="191" spans="1:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:10" ht="55.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A191" s="11" t="s">
         <v>559</v>
       </c>
@@ -10423,7 +10423,7 @@
       <c r="I191" s="11"/>
       <c r="J191" s="20"/>
     </row>
-    <row r="192" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A192" s="11" t="s">
         <v>560</v>
       </c>
@@ -10451,7 +10451,7 @@
       <c r="I192" s="11"/>
       <c r="J192" s="20"/>
     </row>
-    <row r="193" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A193" s="11" t="s">
         <v>562</v>
       </c>
@@ -10479,7 +10479,7 @@
       <c r="I193" s="11"/>
       <c r="J193" s="20"/>
     </row>
-    <row r="194" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A194" s="11" t="s">
         <v>564</v>
       </c>
@@ -10511,7 +10511,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="195" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A195" s="11" t="s">
         <v>567</v>
       </c>
@@ -10543,7 +10543,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="196" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A196" s="11" t="s">
         <v>569</v>
       </c>
@@ -10571,7 +10571,7 @@
       <c r="I196" s="11"/>
       <c r="J196" s="20"/>
     </row>
-    <row r="197" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A197" s="11" t="s">
         <v>571</v>
       </c>
@@ -10599,7 +10599,7 @@
       <c r="I197" s="11"/>
       <c r="J197" s="20"/>
     </row>
-    <row r="198" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A198" s="11" t="s">
         <v>572</v>
       </c>
@@ -10627,7 +10627,7 @@
       <c r="I198" s="11"/>
       <c r="J198" s="20"/>
     </row>
-    <row r="199" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A199" s="11" t="s">
         <v>573</v>
       </c>
@@ -10655,7 +10655,7 @@
       <c r="I199" s="11"/>
       <c r="J199" s="20"/>
     </row>
-    <row r="200" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A200" s="11" t="s">
         <v>574</v>
       </c>
@@ -10685,7 +10685,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="201" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A201" s="11" t="s">
         <v>576</v>
       </c>
@@ -10713,7 +10713,7 @@
       <c r="I201" s="11"/>
       <c r="J201" s="20"/>
     </row>
-    <row r="202" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A202" s="11" t="s">
         <v>578</v>
       </c>
@@ -10741,7 +10741,7 @@
       <c r="I202" s="11"/>
       <c r="J202" s="20"/>
     </row>
-    <row r="203" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A203" s="11" t="s">
         <v>580</v>
       </c>
@@ -10769,7 +10769,7 @@
       <c r="I203" s="11"/>
       <c r="J203" s="20"/>
     </row>
-    <row r="204" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A204" s="11" t="s">
         <v>582</v>
       </c>
@@ -10797,7 +10797,7 @@
       <c r="I204" s="11"/>
       <c r="J204" s="20"/>
     </row>
-    <row r="205" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A205" s="11" t="s">
         <v>584</v>
       </c>
@@ -10825,7 +10825,7 @@
       <c r="I205" s="11"/>
       <c r="J205" s="20"/>
     </row>
-    <row r="206" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A206" s="11" t="s">
         <v>586</v>
       </c>
@@ -10853,7 +10853,7 @@
       <c r="I206" s="11"/>
       <c r="J206" s="20"/>
     </row>
-    <row r="207" spans="1:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:10" ht="55.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A207" s="11" t="s">
         <v>588</v>
       </c>
@@ -10885,7 +10885,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="208" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A208" s="11" t="s">
         <v>591</v>
       </c>
@@ -10917,7 +10917,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="209" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A209" s="11" t="s">
         <v>594</v>
       </c>
@@ -10949,7 +10949,7 @@
         <v>596</v>
       </c>
     </row>
-    <row r="210" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A210" s="11" t="s">
         <v>597</v>
       </c>
@@ -10981,7 +10981,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="211" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A211" s="11" t="s">
         <v>600</v>
       </c>
@@ -11009,7 +11009,7 @@
       <c r="I211" s="11"/>
       <c r="J211" s="20"/>
     </row>
-    <row r="212" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A212" s="11" t="s">
         <v>602</v>
       </c>
@@ -11037,7 +11037,7 @@
       <c r="I212" s="11"/>
       <c r="J212" s="20"/>
     </row>
-    <row r="213" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A213" s="11" t="s">
         <v>604</v>
       </c>
@@ -11065,7 +11065,7 @@
       <c r="I213" s="11"/>
       <c r="J213" s="20"/>
     </row>
-    <row r="214" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A214" s="11" t="s">
         <v>605</v>
       </c>
@@ -11093,7 +11093,7 @@
       <c r="I214" s="11"/>
       <c r="J214" s="20"/>
     </row>
-    <row r="215" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A215" s="11" t="s">
         <v>606</v>
       </c>
@@ -11121,7 +11121,7 @@
       <c r="I215" s="11"/>
       <c r="J215" s="20"/>
     </row>
-    <row r="216" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A216" s="11" t="s">
         <v>607</v>
       </c>
@@ -11149,7 +11149,7 @@
       <c r="I216" s="11"/>
       <c r="J216" s="20"/>
     </row>
-    <row r="217" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A217" s="11" t="s">
         <v>608</v>
       </c>
@@ -11177,7 +11177,7 @@
       <c r="I217" s="11"/>
       <c r="J217" s="20"/>
     </row>
-    <row r="218" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A218" s="11" t="s">
         <v>610</v>
       </c>
@@ -11205,7 +11205,7 @@
       <c r="I218" s="11"/>
       <c r="J218" s="20"/>
     </row>
-    <row r="219" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A219" s="11" t="s">
         <v>612</v>
       </c>
@@ -11233,7 +11233,7 @@
       <c r="I219" s="11"/>
       <c r="J219" s="20"/>
     </row>
-    <row r="220" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A220" s="11" t="s">
         <v>614</v>
       </c>
@@ -11261,7 +11261,7 @@
       <c r="I220" s="11"/>
       <c r="J220" s="20"/>
     </row>
-    <row r="221" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A221" s="11" t="s">
         <v>616</v>
       </c>
@@ -11289,7 +11289,7 @@
       <c r="I221" s="11"/>
       <c r="J221" s="20"/>
     </row>
-    <row r="222" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A222" s="11" t="s">
         <v>618</v>
       </c>
@@ -11317,7 +11317,7 @@
       <c r="I222" s="11"/>
       <c r="J222" s="20"/>
     </row>
-    <row r="223" spans="1:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:10" ht="55.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A223" s="11" t="s">
         <v>620</v>
       </c>
@@ -11349,7 +11349,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="224" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A224" s="11" t="s">
         <v>623</v>
       </c>
@@ -11381,7 +11381,7 @@
         <v>625</v>
       </c>
     </row>
-    <row r="225" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A225" s="11" t="s">
         <v>626</v>
       </c>
@@ -11413,7 +11413,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="226" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A226" s="11" t="s">
         <v>629</v>
       </c>
@@ -11445,7 +11445,7 @@
         <v>631</v>
       </c>
     </row>
-    <row r="227" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A227" s="11" t="s">
         <v>632</v>
       </c>
@@ -11473,7 +11473,7 @@
       <c r="I227" s="11"/>
       <c r="J227" s="20"/>
     </row>
-    <row r="228" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A228" s="11" t="s">
         <v>634</v>
       </c>
@@ -11501,7 +11501,7 @@
       <c r="I228" s="11"/>
       <c r="J228" s="20"/>
     </row>
-    <row r="229" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A229" s="11" t="s">
         <v>636</v>
       </c>
@@ -11529,7 +11529,7 @@
       <c r="I229" s="11"/>
       <c r="J229" s="20"/>
     </row>
-    <row r="230" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A230" s="11" t="s">
         <v>637</v>
       </c>
@@ -11557,7 +11557,7 @@
       <c r="I230" s="11"/>
       <c r="J230" s="20"/>
     </row>
-    <row r="231" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A231" s="11" t="s">
         <v>638</v>
       </c>
@@ -11585,7 +11585,7 @@
       <c r="I231" s="11"/>
       <c r="J231" s="20"/>
     </row>
-    <row r="232" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A232" s="11" t="s">
         <v>639</v>
       </c>
@@ -11613,7 +11613,7 @@
       <c r="I232" s="11"/>
       <c r="J232" s="20"/>
     </row>
-    <row r="233" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A233" s="11" t="s">
         <v>640</v>
       </c>
@@ -11641,7 +11641,7 @@
       <c r="I233" s="11"/>
       <c r="J233" s="20"/>
     </row>
-    <row r="234" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A234" s="11" t="s">
         <v>641</v>
       </c>
@@ -11669,7 +11669,7 @@
       <c r="I234" s="11"/>
       <c r="J234" s="20"/>
     </row>
-    <row r="235" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A235" s="11" t="s">
         <v>643</v>
       </c>
@@ -11697,7 +11697,7 @@
       <c r="I235" s="11"/>
       <c r="J235" s="20"/>
     </row>
-    <row r="236" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A236" s="11" t="s">
         <v>645</v>
       </c>
@@ -11725,7 +11725,7 @@
       <c r="I236" s="11"/>
       <c r="J236" s="20"/>
     </row>
-    <row r="237" spans="1:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:10" ht="55.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A237" s="11" t="s">
         <v>647</v>
       </c>
@@ -11753,7 +11753,7 @@
       <c r="I237" s="11"/>
       <c r="J237" s="20"/>
     </row>
-    <row r="238" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A238" s="11" t="s">
         <v>648</v>
       </c>
@@ -11785,7 +11785,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="239" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A239" s="11" t="s">
         <v>651</v>
       </c>
@@ -11817,7 +11817,7 @@
         <v>653</v>
       </c>
     </row>
-    <row r="240" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A240" s="11" t="s">
         <v>654</v>
       </c>
@@ -11849,7 +11849,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="241" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A241" s="11" t="s">
         <v>657</v>
       </c>
@@ -11877,7 +11877,7 @@
       <c r="I241" s="11"/>
       <c r="J241" s="20"/>
     </row>
-    <row r="242" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A242" s="11" t="s">
         <v>659</v>
       </c>
@@ -11905,7 +11905,7 @@
       <c r="I242" s="11"/>
       <c r="J242" s="20"/>
     </row>
-    <row r="243" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A243" s="11" t="s">
         <v>661</v>
       </c>
@@ -11933,7 +11933,7 @@
       <c r="I243" s="11"/>
       <c r="J243" s="20"/>
     </row>
-    <row r="244" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A244" s="11" t="s">
         <v>662</v>
       </c>
@@ -11961,7 +11961,7 @@
       <c r="I244" s="11"/>
       <c r="J244" s="20"/>
     </row>
-    <row r="245" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A245" s="11" t="s">
         <v>663</v>
       </c>
@@ -11989,7 +11989,7 @@
       <c r="I245" s="11"/>
       <c r="J245" s="20"/>
     </row>
-    <row r="246" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A246" s="11" t="s">
         <v>664</v>
       </c>
@@ -12017,7 +12017,7 @@
       <c r="I246" s="11"/>
       <c r="J246" s="20"/>
     </row>
-    <row r="247" spans="1:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:10" ht="55.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A247" s="11" t="s">
         <v>665</v>
       </c>
@@ -12045,7 +12045,7 @@
       <c r="I247" s="11"/>
       <c r="J247" s="20"/>
     </row>
-    <row r="248" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A248" s="11" t="s">
         <v>666</v>
       </c>
@@ -12073,7 +12073,7 @@
       <c r="I248" s="11"/>
       <c r="J248" s="20"/>
     </row>
-    <row r="249" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A249" s="11" t="s">
         <v>668</v>
       </c>
@@ -12101,7 +12101,7 @@
       <c r="I249" s="11"/>
       <c r="J249" s="20"/>
     </row>
-    <row r="250" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A250" s="11" t="s">
         <v>670</v>
       </c>
@@ -12129,7 +12129,7 @@
       <c r="I250" s="11"/>
       <c r="J250" s="20"/>
     </row>
-    <row r="251" spans="1:10" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:10" ht="82.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A251" s="11" t="s">
         <v>671</v>
       </c>
@@ -12161,7 +12161,7 @@
         <v>673</v>
       </c>
     </row>
-    <row r="252" spans="1:10" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:10" ht="82.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A252" s="11" t="s">
         <v>674</v>
       </c>
@@ -12193,7 +12193,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="253" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A253" s="11" t="s">
         <v>676</v>
       </c>
@@ -12221,7 +12221,7 @@
       <c r="I253" s="11"/>
       <c r="J253" s="20"/>
     </row>
-    <row r="254" spans="1:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:10" ht="55.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A254" s="11" t="s">
         <v>678</v>
       </c>
@@ -12249,7 +12249,7 @@
       <c r="I254" s="11"/>
       <c r="J254" s="20"/>
     </row>
-    <row r="255" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A255" s="11" t="s">
         <v>679</v>
       </c>
@@ -12277,7 +12277,7 @@
       <c r="I255" s="11"/>
       <c r="J255" s="20"/>
     </row>
-    <row r="256" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A256" s="11" t="s">
         <v>680</v>
       </c>
@@ -12350,7 +12350,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F51"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="36" customWidth="1"/>
@@ -12360,7 +12360,7 @@
     <col min="6" max="6" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="29" t="s">
         <v>681</v>
       </c>
@@ -12370,7 +12370,7 @@
       <c r="E1" s="24"/>
       <c r="F1" s="24"/>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="30" t="s">
         <v>682</v>
       </c>
@@ -12380,7 +12380,7 @@
       <c r="E2" s="24"/>
       <c r="F2" s="24"/>
     </row>
-    <row r="5" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>189</v>
       </c>
@@ -12400,7 +12400,7 @@
         <v>686</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="51.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
         <v>86</v>
       </c>
@@ -12420,7 +12420,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="51.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
         <v>86</v>
       </c>
@@ -12440,7 +12440,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="51.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
         <v>86</v>
       </c>
@@ -12460,7 +12460,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
         <v>86</v>
       </c>
@@ -12477,10 +12477,10 @@
         <v>695</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>689</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
         <v>96</v>
       </c>
@@ -12500,7 +12500,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="51.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
         <v>96</v>
       </c>
@@ -12520,7 +12520,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="64.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" ht="64.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
         <v>96</v>
       </c>
@@ -12540,7 +12540,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
         <v>102</v>
       </c>
@@ -12560,7 +12560,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
         <v>102</v>
       </c>
@@ -12580,7 +12580,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
         <v>102</v>
       </c>
@@ -12600,7 +12600,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
         <v>110</v>
       </c>
@@ -12620,7 +12620,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
         <v>110</v>
       </c>
@@ -12640,7 +12640,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="51.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
         <v>110</v>
       </c>
@@ -12660,7 +12660,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
         <v>117</v>
       </c>
@@ -12680,7 +12680,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
         <v>117</v>
       </c>
@@ -12700,7 +12700,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
         <v>117</v>
       </c>
@@ -12720,7 +12720,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
         <v>108</v>
       </c>
@@ -12740,7 +12740,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="13" t="s">
         <v>108</v>
       </c>
@@ -12760,7 +12760,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
         <v>127</v>
       </c>
@@ -12780,7 +12780,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="13" t="s">
         <v>127</v>
       </c>
@@ -12800,7 +12800,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
         <v>132</v>
       </c>
@@ -12820,7 +12820,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="13" t="s">
         <v>132</v>
       </c>
@@ -12840,7 +12840,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="11" t="s">
         <v>132</v>
       </c>
@@ -12860,7 +12860,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="13" t="s">
         <v>125</v>
       </c>
@@ -12880,7 +12880,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="11" t="s">
         <v>125</v>
       </c>
@@ -12900,7 +12900,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="31" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="13" t="s">
         <v>142</v>
       </c>
@@ -12920,7 +12920,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="32" spans="1:6" ht="51.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="11" t="s">
         <v>142</v>
       </c>
@@ -12940,7 +12940,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="13" t="s">
         <v>142</v>
       </c>
@@ -12960,7 +12960,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="11" t="s">
         <v>147</v>
       </c>
@@ -12980,7 +12980,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="13" t="s">
         <v>147</v>
       </c>
@@ -13000,7 +13000,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="36" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="11" t="s">
         <v>147</v>
       </c>
@@ -13020,7 +13020,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="13" t="s">
         <v>152</v>
       </c>
@@ -13040,7 +13040,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="38" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="11" t="s">
         <v>152</v>
       </c>
@@ -13060,7 +13060,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="13" t="s">
         <v>152</v>
       </c>
@@ -13080,7 +13080,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="40" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="11" t="s">
         <v>157</v>
       </c>
@@ -13100,7 +13100,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="13" t="s">
         <v>157</v>
       </c>
@@ -13120,7 +13120,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="11" t="s">
         <v>157</v>
       </c>
@@ -13140,7 +13140,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="43" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="13" t="s">
         <v>165</v>
       </c>
@@ -13160,7 +13160,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="44" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="11" t="s">
         <v>165</v>
       </c>
@@ -13180,7 +13180,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="45" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="13" t="s">
         <v>165</v>
       </c>
@@ -13200,7 +13200,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="46" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="11" t="s">
         <v>171</v>
       </c>
@@ -13220,7 +13220,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="47" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="13" t="s">
         <v>171</v>
       </c>
@@ -13240,7 +13240,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="48" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="11" t="s">
         <v>176</v>
       </c>
@@ -13260,7 +13260,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="49" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="13" t="s">
         <v>176</v>
       </c>
@@ -13280,7 +13280,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="50" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="11" t="s">
         <v>169</v>
       </c>
@@ -13300,7 +13300,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="51" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="13" t="s">
         <v>169</v>
       </c>
@@ -13351,7 +13351,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -13359,7 +13359,7 @@
     <col min="4" max="4" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="29" t="s">
         <v>780</v>
       </c>
@@ -13367,7 +13367,7 @@
       <c r="C1" s="24"/>
       <c r="D1" s="24"/>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="30" t="s">
         <v>781</v>
       </c>
@@ -13375,7 +13375,7 @@
       <c r="C2" s="24"/>
       <c r="D2" s="24"/>
     </row>
-    <row r="4" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>683</v>
       </c>
@@ -13389,7 +13389,7 @@
         <v>784</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="11">
         <v>1</v>
       </c>
@@ -13403,7 +13403,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="13">
         <v>2</v>
       </c>
@@ -13417,7 +13417,7 @@
         <v>788</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="11">
         <v>3</v>
       </c>
@@ -13431,7 +13431,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="13">
         <v>4</v>
       </c>
@@ -13445,7 +13445,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
         <v>5</v>
       </c>
@@ -13459,7 +13459,7 @@
         <v>788</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="13">
         <v>6</v>
       </c>
@@ -13473,7 +13473,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
         <v>7</v>
       </c>
@@ -13487,7 +13487,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="13">
         <v>8</v>
       </c>
@@ -13501,7 +13501,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
         <v>9</v>
       </c>
@@ -13515,7 +13515,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="13">
         <v>10</v>
       </c>
@@ -13529,21 +13529,21 @@
         <v>689</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="25" t="s">
+    <row r="16" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="23" t="s">
         <v>804</v>
       </c>
       <c r="B16" s="24"/>
       <c r="C16" s="24"/>
       <c r="D16" s="24"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="24"/>
       <c r="B17" s="24"/>
       <c r="C17" s="24"/>
       <c r="D17" s="24"/>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="24"/>
       <c r="B18" s="24"/>
       <c r="C18" s="24"/>

</xml_diff>

<commit_message>
T-1011 y T-1012 (HU-001) marcadas como Terminadas en el backlog S1
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S1.xlsx
+++ b/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S1.xlsx
@@ -5354,7 +5354,7 @@
         <v>15</v>
       </c>
       <c r="H16" s="11" t="s">
-        <v>218</v>
+        <v>197</v>
       </c>
       <c r="I16" s="11"/>
       <c r="J16" s="20"/>
@@ -5382,7 +5382,7 @@
         <v>15</v>
       </c>
       <c r="H17" s="11" t="s">
-        <v>218</v>
+        <v>197</v>
       </c>
       <c r="I17" s="11"/>
       <c r="J17" s="20"/>

</xml_diff>